<commit_message>
Unity  - MCP 补充
</commit_message>
<xml_diff>
--- a/config/Config/Data/__enums__.xlsx
+++ b/config/Config/Data/__enums__.xlsx
@@ -337,37 +337,37 @@
     <t>ESkillShowTag</t>
   </si>
   <si>
-    <t>技能展示标签</t>
+    <t>技能分类口吻；Job/Campus/Fusion 仍是机制位</t>
   </si>
   <si>
     <t>Active</t>
   </si>
   <si>
-    <t>主动</t>
+    <t>主动出手</t>
   </si>
   <si>
     <t>Passive</t>
   </si>
   <si>
-    <t>被动</t>
+    <t>挂着就有</t>
   </si>
   <si>
     <t>Job</t>
   </si>
   <si>
-    <t>就业技</t>
+    <t>工牌绝活</t>
   </si>
   <si>
     <t>Campus</t>
   </si>
   <si>
-    <t>校园技</t>
+    <t>课间绝活</t>
   </si>
   <si>
     <t>Fusion</t>
   </si>
   <si>
-    <t>融合技</t>
+    <t>兄弟连招</t>
   </si>
   <si>
     <t>ESkillEffectKind</t>
@@ -481,13 +481,13 @@
     <t>CampusSkill</t>
   </si>
   <si>
-    <t>校园技升级</t>
+    <t>课间绝活升级</t>
   </si>
   <si>
     <t>JobSkill</t>
   </si>
   <si>
-    <t>就业技升级</t>
+    <t>工牌绝活升级</t>
   </si>
   <si>
     <t>Encounter</t>
@@ -505,13 +505,13 @@
     <t>LootSkill</t>
   </si>
   <si>
-    <t>临时掉落技能</t>
+    <t>地摊技</t>
   </si>
   <si>
     <t>Event</t>
   </si>
   <si>
-    <t>龙南事件</t>
+    <t>龙南糗事</t>
   </si>
   <si>
     <t>EAttackForm</t>
@@ -2448,7 +2448,6 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.25"/>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
@@ -2813,7 +2812,6 @@
         <v>105</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25"/>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>8</v>
@@ -3004,7 +3002,6 @@
         <v>8</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25"/>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>8</v>
@@ -3271,7 +3268,6 @@
         <v>8</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25"/>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>8</v>

</xml_diff>